<commit_message>
Rebuild generated files (automatic, from 90caa92)
</commit_message>
<xml_diff>
--- a/spreadsheet/FeasaBULL_Diet_Optimizer.xlsx
+++ b/spreadsheet/FeasaBULL_Diet_Optimizer.xlsx
@@ -52,13 +52,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>49</xdr:colOff>
+                <xdr:colOff>42</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>5</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>2</xdr:col>
-                <xdr:colOff>90</xdr:colOff>
+                <xdr:colOff>55</xdr:colOff>
                 <xdr:row>4</xdr:row>
                 <xdr:rowOff>1</xdr:rowOff>
               </xdr:to>
@@ -85,13 +85,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>49</xdr:colOff>
+                <xdr:colOff>42</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>5</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>2</xdr:col>
-                <xdr:colOff>90</xdr:colOff>
+                <xdr:colOff>55</xdr:colOff>
                 <xdr:row>4</xdr:row>
                 <xdr:rowOff>49</xdr:rowOff>
               </xdr:to>
@@ -118,13 +118,13 @@
             <anchor moveWithCells="false" sizeWithCells="false">
               <xdr:from>
                 <xdr:col>1</xdr:col>
-                <xdr:colOff>49</xdr:colOff>
+                <xdr:colOff>42</xdr:colOff>
                 <xdr:row>0</xdr:row>
                 <xdr:rowOff>5</xdr:rowOff>
               </xdr:from>
               <xdr:to>
                 <xdr:col>2</xdr:col>
-                <xdr:colOff>90</xdr:colOff>
+                <xdr:colOff>55</xdr:colOff>
                 <xdr:row>4</xdr:row>
                 <xdr:rowOff>19</xdr:rowOff>
               </xdr:to>
@@ -139,7 +139,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1268" uniqueCount="825">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1273" uniqueCount="829">
   <si>
     <t xml:space="preserve">FeasaBULL Diet Planner — person in, cheapest balanced day out</t>
   </si>
@@ -1936,6 +1936,18 @@
   </si>
   <si>
     <t xml:space="preserve">All foods except pork</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nut-Free</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No peanuts or tree nuts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20,66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peanut butter; Almonds</t>
   </si>
   <si>
     <t xml:space="preserve">Low-Carb sets carbohydrate below the AMDR range (45–65%) on purpose; High-Protein sits at the top of the AMDR protein range.</t>
@@ -3704,7 +3716,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L72"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
@@ -3933,7 +3945,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="16" t="s">
         <v>41</v>
       </c>
@@ -4473,7 +4485,7 @@
         <v>82</v>
       </c>
       <c r="C37" s="29" t="str">
-        <f aca="false">INDEX(Diets!$B$5:$B$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))</f>
+        <f aca="false">INDEX(Diets!$B$5:$B$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))</f>
         <v>USDA Acceptable Macronutrient Distribution Ranges; all foods allowed</v>
       </c>
     </row>
@@ -5332,7 +5344,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C36" type="list">
-      <formula1>Diets!$A$5:$A$12</formula1>
+      <formula1>Diets!$A$5:$A$13</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C39" type="list">
@@ -5356,7 +5368,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J29"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="2" style="0" width="12"/>
@@ -5594,7 +5606,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="s">
         <v>73</v>
       </c>
@@ -5808,7 +5820,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AW76"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
@@ -6077,7 +6089,7 @@
         <v>0</v>
       </c>
       <c r="Z6" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S6:Y6,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A6&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S6:Y6,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A6&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA6" s="44" t="n">
@@ -6225,7 +6237,7 @@
         <v>0</v>
       </c>
       <c r="Z7" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S7:Y7,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A7&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S7:Y7,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A7&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA7" s="44" t="n">
@@ -6368,7 +6380,7 @@
         <v>0</v>
       </c>
       <c r="Z8" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S8:Y8,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A8&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S8:Y8,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A8&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA8" s="44" t="n">
@@ -6511,7 +6523,7 @@
         <v>0</v>
       </c>
       <c r="Z9" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S9:Y9,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A9&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S9:Y9,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A9&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA9" s="44" t="n">
@@ -6652,7 +6664,7 @@
         <v>0</v>
       </c>
       <c r="Z10" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S10:Y10,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A10&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S10:Y10,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A10&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA10" s="44" t="n">
@@ -6800,7 +6812,7 @@
         <v>0</v>
       </c>
       <c r="Z11" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S11:Y11,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A11&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S11:Y11,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A11&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA11" s="44" t="n">
@@ -6948,7 +6960,7 @@
         <v>0</v>
       </c>
       <c r="Z12" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S12:Y12,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A12&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S12:Y12,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A12&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA12" s="44" t="n">
@@ -7096,7 +7108,7 @@
         <v>0</v>
       </c>
       <c r="Z13" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S13:Y13,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A13&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S13:Y13,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A13&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA13" s="44" t="n">
@@ -7244,7 +7256,7 @@
         <v>0</v>
       </c>
       <c r="Z14" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S14:Y14,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A14&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S14:Y14,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A14&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA14" s="44" t="n">
@@ -7394,7 +7406,7 @@
         <v>0</v>
       </c>
       <c r="Z15" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S15:Y15,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A15&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S15:Y15,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A15&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA15" s="44" t="n">
@@ -7542,7 +7554,7 @@
         <v>0</v>
       </c>
       <c r="Z16" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S16:Y16,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A16&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S16:Y16,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A16&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA16" s="44" t="n">
@@ -7683,7 +7695,7 @@
         <v>0</v>
       </c>
       <c r="Z17" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S17:Y17,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A17&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S17:Y17,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A17&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA17" s="44" t="n">
@@ -7826,7 +7838,7 @@
         <v>0</v>
       </c>
       <c r="Z18" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S18:Y18,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A18&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S18:Y18,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A18&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA18" s="44" t="n">
@@ -7967,7 +7979,7 @@
         <v>0</v>
       </c>
       <c r="Z19" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S19:Y19,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A19&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S19:Y19,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A19&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA19" s="44" t="n">
@@ -8108,7 +8120,7 @@
         <v>0</v>
       </c>
       <c r="Z20" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S20:Y20,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A20&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S20:Y20,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A20&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA20" s="44" t="n">
@@ -8256,7 +8268,7 @@
         <v>0</v>
       </c>
       <c r="Z21" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S21:Y21,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A21&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S21:Y21,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A21&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA21" s="44" t="n">
@@ -8397,7 +8409,7 @@
         <v>0</v>
       </c>
       <c r="Z22" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S22:Y22,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A22&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S22:Y22,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A22&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA22" s="44" t="n">
@@ -8540,7 +8552,7 @@
         <v>0</v>
       </c>
       <c r="Z23" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S23:Y23,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A23&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S23:Y23,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A23&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA23" s="44" t="n">
@@ -8683,7 +8695,7 @@
         <v>0</v>
       </c>
       <c r="Z24" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S24:Y24,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A24&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S24:Y24,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A24&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA24" s="44" t="n">
@@ -8824,7 +8836,7 @@
         <v>0</v>
       </c>
       <c r="Z25" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S25:Y25,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A25&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S25:Y25,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A25&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA25" s="44" t="n">
@@ -8970,7 +8982,7 @@
         <v>0</v>
       </c>
       <c r="Z26" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S26:Y26,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A26&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S26:Y26,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A26&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA26" s="44" t="n">
@@ -9111,7 +9123,7 @@
         <v>0</v>
       </c>
       <c r="Z27" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S27:Y27,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A27&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S27:Y27,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A27&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA27" s="44" t="n">
@@ -9252,7 +9264,7 @@
         <v>0</v>
       </c>
       <c r="Z28" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S28:Y28,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A28&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S28:Y28,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A28&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA28" s="44" t="n">
@@ -9393,7 +9405,7 @@
         <v>0</v>
       </c>
       <c r="Z29" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S29:Y29,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A29&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S29:Y29,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A29&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA29" s="44" t="n">
@@ -9532,7 +9544,7 @@
         <v>0</v>
       </c>
       <c r="Z30" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S30:Y30,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A30&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S30:Y30,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A30&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA30" s="44" t="n">
@@ -9680,7 +9692,7 @@
         <v>0</v>
       </c>
       <c r="Z31" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S31:Y31,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A31&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S31:Y31,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A31&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA31" s="44" t="n">
@@ -9828,7 +9840,7 @@
         <v>0</v>
       </c>
       <c r="Z32" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S32:Y32,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A32&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S32:Y32,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A32&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA32" s="44" t="n">
@@ -9976,7 +9988,7 @@
         <v>0</v>
       </c>
       <c r="Z33" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S33:Y33,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A33&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S33:Y33,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A33&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA33" s="44" t="n">
@@ -10117,7 +10129,7 @@
         <v>0</v>
       </c>
       <c r="Z34" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S34:Y34,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A34&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S34:Y34,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A34&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA34" s="44" t="n">
@@ -10258,7 +10270,7 @@
         <v>0</v>
       </c>
       <c r="Z35" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S35:Y35,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A35&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S35:Y35,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A35&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA35" s="44" t="n">
@@ -10401,7 +10413,7 @@
         <v>1</v>
       </c>
       <c r="Z36" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S36:Y36,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A36&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S36:Y36,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A36&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA36" s="44" t="n">
@@ -10542,7 +10554,7 @@
         <v>0</v>
       </c>
       <c r="Z37" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S37:Y37,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A37&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S37:Y37,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A37&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA37" s="44" t="n">
@@ -10683,7 +10695,7 @@
         <v>0</v>
       </c>
       <c r="Z38" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S38:Y38,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A38&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S38:Y38,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A38&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA38" s="44" t="n">
@@ -10826,7 +10838,7 @@
         <v>0</v>
       </c>
       <c r="Z39" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S39:Y39,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A39&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S39:Y39,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A39&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA39" s="44" t="n">
@@ -10969,7 +10981,7 @@
         <v>1</v>
       </c>
       <c r="Z40" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S40:Y40,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A40&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S40:Y40,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A40&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA40" s="44" t="n">
@@ -11110,7 +11122,7 @@
         <v>0</v>
       </c>
       <c r="Z41" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S41:Y41,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A41&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S41:Y41,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A41&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA41" s="44" t="n">
@@ -11251,7 +11263,7 @@
         <v>1</v>
       </c>
       <c r="Z42" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S42:Y42,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A42&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S42:Y42,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A42&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA42" s="44" t="n">
@@ -11401,7 +11413,7 @@
         <v>1</v>
       </c>
       <c r="Z43" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S43:Y43,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A43&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S43:Y43,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A43&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA43" s="44" t="n">
@@ -11549,7 +11561,7 @@
         <v>1</v>
       </c>
       <c r="Z44" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S44:Y44,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A44&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S44:Y44,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A44&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA44" s="44" t="n">
@@ -11697,7 +11709,7 @@
         <v>0</v>
       </c>
       <c r="Z45" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S45:Y45,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A45&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S45:Y45,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A45&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA45" s="44" t="n">
@@ -11840,7 +11852,7 @@
         <v>1</v>
       </c>
       <c r="Z46" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S46:Y46,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A46&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S46:Y46,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A46&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA46" s="44" t="n">
@@ -11981,7 +11993,7 @@
         <v>1</v>
       </c>
       <c r="Z47" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S47:Y47,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A47&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S47:Y47,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A47&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA47" s="44" t="n">
@@ -12124,7 +12136,7 @@
         <v>0</v>
       </c>
       <c r="Z48" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S48:Y48,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A48&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S48:Y48,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A48&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA48" s="44" t="n">
@@ -12272,7 +12284,7 @@
         <v>0</v>
       </c>
       <c r="Z49" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S49:Y49,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A49&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S49:Y49,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A49&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA49" s="44" t="n">
@@ -12413,7 +12425,7 @@
         <v>0</v>
       </c>
       <c r="Z50" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S50:Y50,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A50&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S50:Y50,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A50&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA50" s="44" t="n">
@@ -12554,7 +12566,7 @@
         <v>0</v>
       </c>
       <c r="Z51" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S51:Y51,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A51&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S51:Y51,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A51&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA51" s="44" t="n">
@@ -12704,7 +12716,7 @@
         <v>0</v>
       </c>
       <c r="Z52" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S52:Y52,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A52&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S52:Y52,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A52&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA52" s="44" t="n">
@@ -12845,7 +12857,7 @@
         <v>0</v>
       </c>
       <c r="Z53" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S53:Y53,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A53&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S53:Y53,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A53&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA53" s="44" t="n">
@@ -12986,7 +12998,7 @@
         <v>0</v>
       </c>
       <c r="Z54" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S54:Y54,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A54&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S54:Y54,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A54&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA54" s="44" t="n">
@@ -13127,7 +13139,7 @@
         <v>0</v>
       </c>
       <c r="Z55" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S55:Y55,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A55&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S55:Y55,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A55&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA55" s="44" t="n">
@@ -13277,7 +13289,7 @@
         <v>0</v>
       </c>
       <c r="Z56" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S56:Y56,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A56&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S56:Y56,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A56&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA56" s="44" t="n">
@@ -13418,7 +13430,7 @@
         <v>0</v>
       </c>
       <c r="Z57" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S57:Y57,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A57&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S57:Y57,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A57&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA57" s="44" t="n">
@@ -13566,7 +13578,7 @@
         <v>0</v>
       </c>
       <c r="Z58" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S58:Y58,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A58&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S58:Y58,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A58&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA58" s="44" t="n">
@@ -13707,7 +13719,7 @@
         <v>0</v>
       </c>
       <c r="Z59" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S59:Y59,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A59&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S59:Y59,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A59&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA59" s="44" t="n">
@@ -13848,7 +13860,7 @@
         <v>0</v>
       </c>
       <c r="Z60" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S60:Y60,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A60&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S60:Y60,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A60&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA60" s="44" t="n">
@@ -13989,7 +14001,7 @@
         <v>0</v>
       </c>
       <c r="Z61" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S61:Y61,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A61&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S61:Y61,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A61&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA61" s="44" t="n">
@@ -14132,7 +14144,7 @@
         <v>0</v>
       </c>
       <c r="Z62" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S62:Y62,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A62&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S62:Y62,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A62&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA62" s="44" t="n">
@@ -14275,7 +14287,7 @@
         <v>0</v>
       </c>
       <c r="Z63" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S63:Y63,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A63&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S63:Y63,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A63&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA63" s="44" t="n">
@@ -14416,7 +14428,7 @@
         <v>0</v>
       </c>
       <c r="Z64" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S64:Y64,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A64&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S64:Y64,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A64&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA64" s="44" t="n">
@@ -14566,7 +14578,7 @@
         <v>0</v>
       </c>
       <c r="Z65" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S65:Y65,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A65&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S65:Y65,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A65&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA65" s="44" t="n">
@@ -14709,7 +14721,7 @@
         <v>0</v>
       </c>
       <c r="Z66" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S66:Y66,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A66&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S66:Y66,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A66&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA66" s="44" t="n">
@@ -14859,7 +14871,7 @@
         <v>0</v>
       </c>
       <c r="Z67" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S67:Y67,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A67&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S67:Y67,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A67&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA67" s="44" t="n">
@@ -15000,7 +15012,7 @@
         <v>0</v>
       </c>
       <c r="Z68" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S68:Y68,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A68&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S68:Y68,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A68&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA68" s="44" t="n">
@@ -15141,7 +15153,7 @@
         <v>0</v>
       </c>
       <c r="Z69" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S69:Y69,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A69&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S69:Y69,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A69&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA69" s="44" t="n">
@@ -15284,7 +15296,7 @@
         <v>0</v>
       </c>
       <c r="Z70" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S70:Y70,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A70&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S70:Y70,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A70&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA70" s="44" t="n">
@@ -15427,7 +15439,7 @@
         <v>0</v>
       </c>
       <c r="Z71" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S71:Y71,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A71&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S71:Y71,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A71&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA71" s="44" t="n">
@@ -15568,7 +15580,7 @@
         <v>0</v>
       </c>
       <c r="Z72" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S72:Y72,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A72&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S72:Y72,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A72&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA72" s="44" t="n">
@@ -15716,7 +15728,7 @@
         <v>1</v>
       </c>
       <c r="Z73" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S73:Y73,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A73&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S73:Y73,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A73&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA73" s="44" t="n">
@@ -15859,7 +15871,7 @@
         <v>1</v>
       </c>
       <c r="Z74" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S74:Y74,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A74&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S74:Y74,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A74&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA74" s="44" t="n">
@@ -16009,7 +16021,7 @@
         <v>0</v>
       </c>
       <c r="Z75" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S75:Y75,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A75&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S75:Y75,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A75&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA75" s="44" t="n">
@@ -16159,7 +16171,7 @@
         <v>0</v>
       </c>
       <c r="Z76" s="43" t="n">
-        <f aca="false">SUMPRODUCT(S76:Y76,INDEX(Diets!$I$5:$O$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0),0))+ISNUMBER(SEARCH(","&amp;A76&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))," ","")&amp;","))*1</f>
+        <f aca="false">SUMPRODUCT(S76:Y76,INDEX(Diets!$I$5:$O$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0),0))+ISNUMBER(SEARCH(","&amp;A76&amp;",",","&amp;SUBSTITUTE(INDEX(Diets!$P$5:$P$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))," ","")&amp;","))*1</f>
         <v>0</v>
       </c>
       <c r="AA76" s="44" t="n">
@@ -16257,8 +16269,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:Q16"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="60"/>
@@ -16428,7 +16440,7 @@
       <c r="P6" s="59"/>
       <c r="Q6" s="29"/>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
         <v>587</v>
       </c>
@@ -16722,14 +16734,67 @@
       <c r="P12" s="59"/>
       <c r="Q12" s="29"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="s">
         <v>599</v>
+      </c>
+      <c r="B13" s="29" t="s">
+        <v>600</v>
+      </c>
+      <c r="C13" s="31" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D13" s="31" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E13" s="31" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="F13" s="31" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G13" s="31" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H13" s="31" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="I13" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="59" t="s">
+        <v>601</v>
+      </c>
+      <c r="Q13" s="29" t="s">
+        <v>602</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>600</v>
+        <v>603</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>604</v>
       </c>
     </row>
   </sheetData>
@@ -16749,7 +16814,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:BX199"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
@@ -16759,17 +16824,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="15" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="C4" s="60" t="str">
         <f aca="false">Planner!$C$36</f>
@@ -16778,57 +16843,57 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="16" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="4" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="C8" s="61" t="n">
-        <f aca="false">INDEX(Diets!$C$5:$C$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))</f>
+        <f aca="false">INDEX(Diets!$C$5:$C$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))</f>
         <v>0.1</v>
       </c>
       <c r="D8" s="61" t="n">
-        <f aca="false">INDEX(Diets!$D$5:$D$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))</f>
+        <f aca="false">INDEX(Diets!$D$5:$D$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))</f>
         <v>0.35</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="4" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="C9" s="61" t="n">
-        <f aca="false">INDEX(Diets!$E$5:$E$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))</f>
+        <f aca="false">INDEX(Diets!$E$5:$E$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))</f>
         <v>0.45</v>
       </c>
       <c r="D9" s="61" t="n">
-        <f aca="false">INDEX(Diets!$F$5:$F$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))</f>
+        <f aca="false">INDEX(Diets!$F$5:$F$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))</f>
         <v>0.65</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="4" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="C10" s="61" t="n">
-        <f aca="false">INDEX(Diets!$G$5:$G$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))</f>
+        <f aca="false">INDEX(Diets!$G$5:$G$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))</f>
         <v>0.2</v>
       </c>
       <c r="D10" s="61" t="n">
-        <f aca="false">INDEX(Diets!$H$5:$H$12,MATCH(Planner!$C$36,Diets!$A$5:$A$12,0))</f>
+        <f aca="false">INDEX(Diets!$H$5:$H$13,MATCH(Planner!$C$36,Diets!$A$5:$A$13,0))</f>
         <v>0.35</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17122,7 +17187,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="62" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="F14" s="70" t="n">
         <f aca="false">'Food Data'!M6</f>
@@ -17411,7 +17476,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="62" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="F15" s="71" t="n">
         <f aca="false">'Food Data'!N6*'Food Data'!P6/100*'Food Data'!AA6</f>
@@ -17700,7 +17765,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="62" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="F16" s="71" t="n">
         <f aca="false">MIN(F15,N('Food Data'!R6)*'Food Data'!N6/100)</f>
@@ -17989,7 +18054,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="62" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="F17" s="72" t="n">
         <f aca="false">'Food Data'!AA6</f>
@@ -18278,7 +18343,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -21462,7 +21527,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22623,21 +22688,21 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="16" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="C39" s="16" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="D39" s="16" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="E39" s="16" t="s">
         <v>16</v>
@@ -22929,10 +22994,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="B40" s="75" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="C40" s="76" t="n">
         <f aca="false">Planner!$E$16*(1-Planner!$C$42)</f>
@@ -23233,10 +23298,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="B41" s="75" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="C41" s="76" t="n">
         <f aca="false">N(Planner!$E$17)</f>
@@ -23536,10 +23601,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="B42" s="75" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="C42" s="78" t="n">
         <v>0</v>
@@ -23838,10 +23903,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="B43" s="75" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="C43" s="78" t="n">
         <v>0</v>
@@ -24140,10 +24205,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="B44" s="75" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="C44" s="78" t="n">
         <v>0</v>
@@ -24442,10 +24507,10 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="B45" s="75" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="C45" s="76" t="n">
         <f aca="false">N(Planner!$E$18)</f>
@@ -24745,10 +24810,10 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="B46" s="75" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="C46" s="76" t="n">
         <f aca="false">N(Planner!$E$19)</f>
@@ -25048,10 +25113,10 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="B47" s="75" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="C47" s="76" t="n">
         <f aca="false">N(Planner!$E$20)</f>
@@ -25351,10 +25416,10 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="B48" s="75" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="C48" s="76" t="n">
         <f aca="false">N(Planner!$E$21)</f>
@@ -25654,10 +25719,10 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="B49" s="75" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="C49" s="76" t="n">
         <f aca="false">N(Planner!$E$22)</f>
@@ -25957,10 +26022,10 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="B50" s="75" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="C50" s="76" t="n">
         <f aca="false">Planner!$E$16*Planner!$C$45</f>
@@ -26260,10 +26325,10 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
       <c r="B51" s="75" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="C51" s="76" t="n">
         <f aca="false">Planner!$E$16*Planner!$C$46</f>
@@ -26563,10 +26628,10 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="B52" s="75" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="C52" s="76" t="n">
         <f aca="false">Planner!$E$16*Planner!$C$47</f>
@@ -26866,10 +26931,10 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="B53" s="75" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="C53" s="76" t="n">
         <f aca="false">Planner!$E$16*Planner!$C$48</f>
@@ -27169,10 +27234,10 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="s">
+        <v>643</v>
+      </c>
+      <c r="B54" s="75" t="s">
         <v>639</v>
-      </c>
-      <c r="B54" s="75" t="s">
-        <v>635</v>
       </c>
       <c r="C54" s="78" t="n">
         <v>0</v>
@@ -27471,10 +27536,10 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="B55" s="75" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="C55" s="78" t="n">
         <v>0</v>
@@ -27773,10 +27838,10 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="4" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="B56" s="75" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="C56" s="78" t="n">
         <v>0</v>
@@ -28075,10 +28140,10 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
       <c r="B57" s="75" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="C57" s="76" t="n">
         <f aca="false">Planner!$C$49</f>
@@ -28378,10 +28443,10 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="4" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="B58" s="75" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="C58" s="76" t="n">
         <f aca="false">Planner!$C$50</f>
@@ -28681,10 +28746,10 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="B59" s="75" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="C59" s="76" t="n">
         <f aca="false">Planner!$E$16*(1+Planner!$C$42)</f>
@@ -28984,10 +29049,10 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
       <c r="B60" s="75" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="C60" s="78" t="n">
         <v>0</v>
@@ -29286,10 +29351,10 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="4" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="B61" s="75" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="C61" s="78" t="n">
         <v>0</v>
@@ -29588,10 +29653,10 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="B62" s="75" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="C62" s="78" t="n">
         <v>0</v>
@@ -29890,10 +29955,10 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="B63" s="75" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="C63" s="76" t="n">
         <f aca="false">N(Planner!$E$23)</f>
@@ -30193,10 +30258,10 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="B64" s="75" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="C64" s="76" t="n">
         <f aca="false">IF(Planner!$E$24="",1000000,Planner!$E$24)</f>
@@ -30496,10 +30561,10 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="4" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="B65" s="75" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="C65" s="76" t="n">
         <f aca="false">Planner!$E$16*Planner!$D$45</f>
@@ -30799,10 +30864,10 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="B66" s="75" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="C66" s="76" t="n">
         <f aca="false">Planner!$E$16*Planner!$D$46</f>
@@ -31102,10 +31167,10 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="4" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
       <c r="B67" s="75" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="C67" s="76" t="n">
         <f aca="false">Planner!$E$16*Planner!$D$47</f>
@@ -31405,10 +31470,10 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="4" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
       <c r="B68" s="75" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="C68" s="76" t="n">
         <f aca="false">Planner!$E$16*Planner!$D$48</f>
@@ -31708,10 +31773,10 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="4" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
       <c r="B69" s="75" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="C69" s="76" t="n">
         <f aca="false">Planner!$C$51</f>
@@ -32011,10 +32076,10 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="4" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="B70" s="75" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="C70" s="76" t="n">
         <f aca="false">Planner!$C$52</f>
@@ -32314,10 +32379,10 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="4" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="B71" s="75" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="C71" s="76" t="n">
         <f aca="false">Planner!$C$53</f>
@@ -32617,10 +32682,10 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="4" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="B72" s="75" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="C72" s="76" t="n">
         <f aca="false">Planner!$C$54</f>
@@ -32920,10 +32985,10 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="4" t="s">
+        <v>667</v>
+      </c>
+      <c r="B73" s="75" t="s">
         <v>663</v>
-      </c>
-      <c r="B73" s="75" t="s">
-        <v>659</v>
       </c>
       <c r="C73" s="76" t="n">
         <f aca="false">Planner!$C$55</f>
@@ -33223,10 +33288,10 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="4" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="B74" s="75" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="C74" s="76" t="n">
         <f aca="false">Planner!$C$56</f>
@@ -33526,10 +33591,10 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="4" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="B75" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C75" s="78" t="n">
         <v>0</v>
@@ -33828,10 +33893,10 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="4" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
       <c r="B76" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C76" s="78" t="n">
         <v>0</v>
@@ -34130,10 +34195,10 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="4" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="B77" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C77" s="78" t="n">
         <v>0</v>
@@ -34432,10 +34497,10 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="4" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="B78" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C78" s="78" t="n">
         <v>0</v>
@@ -34734,10 +34799,10 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="4" t="s">
+        <v>674</v>
+      </c>
+      <c r="B79" s="75" t="s">
         <v>670</v>
-      </c>
-      <c r="B79" s="75" t="s">
-        <v>666</v>
       </c>
       <c r="C79" s="78" t="n">
         <v>0</v>
@@ -35036,10 +35101,10 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="4" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="B80" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C80" s="78" t="n">
         <v>0</v>
@@ -35338,10 +35403,10 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="4" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="B81" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C81" s="78" t="n">
         <v>0</v>
@@ -35640,10 +35705,10 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="4" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="B82" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C82" s="78" t="n">
         <v>0</v>
@@ -35942,10 +36007,10 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="4" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="B83" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C83" s="78" t="n">
         <v>0</v>
@@ -36244,10 +36309,10 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="4" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
       <c r="B84" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C84" s="78" t="n">
         <v>0</v>
@@ -36546,10 +36611,10 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="4" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="B85" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C85" s="78" t="n">
         <v>0</v>
@@ -36848,10 +36913,10 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="4" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
       <c r="B86" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C86" s="78" t="n">
         <v>0</v>
@@ -37150,10 +37215,10 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="4" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
       <c r="B87" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C87" s="78" t="n">
         <v>0</v>
@@ -37452,10 +37517,10 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="4" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
       <c r="B88" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C88" s="78" t="n">
         <v>0</v>
@@ -37754,10 +37819,10 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="4" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
       <c r="B89" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C89" s="78" t="n">
         <v>0</v>
@@ -38056,10 +38121,10 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="4" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="B90" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C90" s="78" t="n">
         <v>0</v>
@@ -38358,10 +38423,10 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="4" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="B91" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C91" s="78" t="n">
         <v>0</v>
@@ -38660,10 +38725,10 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="4" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="B92" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C92" s="78" t="n">
         <v>0</v>
@@ -38962,10 +39027,10 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="4" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="B93" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C93" s="78" t="n">
         <v>0</v>
@@ -39264,10 +39329,10 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="4" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="B94" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C94" s="78" t="n">
         <v>0</v>
@@ -39566,10 +39631,10 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="4" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="B95" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C95" s="78" t="n">
         <v>0</v>
@@ -39868,10 +39933,10 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="4" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="B96" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C96" s="78" t="n">
         <v>0</v>
@@ -40170,10 +40235,10 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="4" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="B97" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C97" s="78" t="n">
         <v>0</v>
@@ -40472,10 +40537,10 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="4" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="B98" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C98" s="78" t="n">
         <v>0</v>
@@ -40774,10 +40839,10 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="4" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="B99" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C99" s="78" t="n">
         <v>0</v>
@@ -41076,10 +41141,10 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="4" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="B100" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C100" s="78" t="n">
         <v>0</v>
@@ -41378,10 +41443,10 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="4" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="B101" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C101" s="78" t="n">
         <v>0</v>
@@ -41680,10 +41745,10 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="4" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="B102" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C102" s="78" t="n">
         <v>0</v>
@@ -41982,10 +42047,10 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="4" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="B103" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C103" s="78" t="n">
         <v>0</v>
@@ -42284,10 +42349,10 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="4" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
       <c r="B104" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C104" s="78" t="n">
         <v>0</v>
@@ -42586,10 +42651,10 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="4" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="B105" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C105" s="78" t="n">
         <v>0</v>
@@ -42888,10 +42953,10 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="4" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="B106" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C106" s="78" t="n">
         <v>0</v>
@@ -43190,10 +43255,10 @@
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="4" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
       <c r="B107" s="75" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C107" s="78" t="n">
         <v>0</v>
@@ -43492,7 +43557,7 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="3" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -43503,49 +43568,49 @@
         <v>157</v>
       </c>
       <c r="C111" s="16" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="D111" s="16" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
       <c r="E111" s="16" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
       <c r="F111" s="16" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="G111" s="16" t="s">
         <v>68</v>
       </c>
       <c r="H111" s="16" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="I111" s="16" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
       <c r="J111" s="16" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
       <c r="K111" s="16" t="s">
-        <v>707</v>
+        <v>711</v>
       </c>
       <c r="L111" s="16" t="s">
-        <v>708</v>
+        <v>712</v>
       </c>
       <c r="M111" s="16" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="N111" s="16" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="O111" s="16" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="P111" s="16" t="s">
-        <v>712</v>
+        <v>716</v>
       </c>
       <c r="Q111" s="16" t="s">
-        <v>713</v>
+        <v>717</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48378,7 +48443,7 @@
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B184" s="62" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="C184" s="82" t="n">
         <f aca="false" t="array" ref="C184:C184">MMULT(F14:BX14,C112:C182)</f>
@@ -48396,7 +48461,7 @@
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="3" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48404,7 +48469,7 @@
         <v>28</v>
       </c>
       <c r="C188" s="16" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="D188" s="16" t="s">
         <v>66</v>
@@ -48665,22 +48730,22 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K109"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L109"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="3" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>717</v>
+        <v>721</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>718</v>
+        <v>722</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -48715,7 +48780,10 @@
         <v>597</v>
       </c>
       <c r="K5" s="16" t="s">
-        <v>719</v>
+        <v>599</v>
+      </c>
+      <c r="L5" s="16" t="s">
+        <v>723</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48753,6 +48821,9 @@
       <c r="K6" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L6" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="n">
@@ -48787,6 +48858,9 @@
         <v>0</v>
       </c>
       <c r="K7" s="85" t="n">
+        <v>0.409277153</v>
+      </c>
+      <c r="L7" s="85" t="n">
         <v>0</v>
       </c>
     </row>
@@ -48825,6 +48899,9 @@
       <c r="K8" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L8" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
@@ -48859,6 +48936,9 @@
         <v>0</v>
       </c>
       <c r="K9" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="85" t="n">
         <v>1.12</v>
       </c>
     </row>
@@ -48897,6 +48977,9 @@
       <c r="K10" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L10" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="n">
@@ -48933,6 +49016,9 @@
       <c r="K11" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L11" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="n">
@@ -48967,6 +49053,9 @@
         <v>0</v>
       </c>
       <c r="K12" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="85" t="n">
         <v>1.13</v>
       </c>
     </row>
@@ -49005,6 +49094,9 @@
       <c r="K13" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L13" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="n">
@@ -49041,6 +49133,9 @@
       <c r="K14" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L14" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="n">
@@ -49077,6 +49172,9 @@
       <c r="K15" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L15" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="n">
@@ -49113,6 +49211,9 @@
       <c r="K16" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L16" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="n">
@@ -49149,6 +49250,9 @@
       <c r="K17" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L17" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="n">
@@ -49185,6 +49289,9 @@
       <c r="K18" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L18" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="n">
@@ -49221,6 +49328,9 @@
       <c r="K19" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L19" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="n">
@@ -49257,6 +49367,9 @@
       <c r="K20" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L20" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="n">
@@ -49291,6 +49404,9 @@
         <v>1.263755108</v>
       </c>
       <c r="K21" s="85" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L21" s="85" t="n">
         <v>0</v>
       </c>
     </row>
@@ -49329,6 +49445,9 @@
       <c r="K22" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L22" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="n">
@@ -49365,6 +49484,9 @@
       <c r="K23" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L23" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="n">
@@ -49401,6 +49523,9 @@
       <c r="K24" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L24" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="n">
@@ -49437,6 +49562,9 @@
       <c r="K25" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L25" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="n">
@@ -49471,6 +49599,9 @@
         <v>1.44</v>
       </c>
       <c r="K26" s="85" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="L26" s="85" t="n">
         <v>0</v>
       </c>
     </row>
@@ -49509,6 +49640,9 @@
       <c r="K27" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L27" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="n">
@@ -49543,6 +49677,9 @@
         <v>4.702468822</v>
       </c>
       <c r="K28" s="85" t="n">
+        <v>4.659972785</v>
+      </c>
+      <c r="L28" s="85" t="n">
         <v>0</v>
       </c>
     </row>
@@ -49581,6 +49718,9 @@
       <c r="K29" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L29" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="n">
@@ -49617,6 +49757,9 @@
       <c r="K30" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L30" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="n">
@@ -49653,6 +49796,9 @@
       <c r="K31" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L31" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="n">
@@ -49687,6 +49833,9 @@
         <v>0</v>
       </c>
       <c r="K32" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="85" t="n">
         <v>0.57</v>
       </c>
     </row>
@@ -49723,6 +49872,9 @@
         <v>0</v>
       </c>
       <c r="K33" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="85" t="n">
         <v>0.28</v>
       </c>
     </row>
@@ -49761,6 +49913,9 @@
       <c r="K34" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L34" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="n">
@@ -49797,6 +49952,9 @@
       <c r="K35" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L35" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="n">
@@ -49831,6 +49989,9 @@
         <v>0</v>
       </c>
       <c r="K36" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" s="85" t="n">
         <v>0.94</v>
       </c>
     </row>
@@ -49867,6 +50028,9 @@
         <v>1.562933795</v>
       </c>
       <c r="K37" s="85" t="n">
+        <v>1.361796895</v>
+      </c>
+      <c r="L37" s="85" t="n">
         <v>0</v>
       </c>
     </row>
@@ -49905,6 +50069,9 @@
       <c r="K38" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L38" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="n">
@@ -49941,6 +50108,9 @@
       <c r="K39" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L39" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="n">
@@ -49977,6 +50147,9 @@
       <c r="K40" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L40" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="n">
@@ -50013,6 +50186,9 @@
       <c r="K41" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L41" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="n">
@@ -50047,6 +50223,9 @@
         <v>0.029924272</v>
       </c>
       <c r="K42" s="85" t="n">
+        <v>0.448497837</v>
+      </c>
+      <c r="L42" s="85" t="n">
         <v>0</v>
       </c>
     </row>
@@ -50083,6 +50262,9 @@
         <v>0</v>
       </c>
       <c r="K43" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" s="85" t="n">
         <v>1.7</v>
       </c>
     </row>
@@ -50119,6 +50301,9 @@
         <v>0</v>
       </c>
       <c r="K44" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" s="85" t="n">
         <v>1.12</v>
       </c>
     </row>
@@ -50155,6 +50340,9 @@
         <v>1.84</v>
       </c>
       <c r="K45" s="85" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="L45" s="85" t="n">
         <v>0</v>
       </c>
     </row>
@@ -50193,6 +50381,9 @@
       <c r="K46" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L46" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="n">
@@ -50229,6 +50420,9 @@
       <c r="K47" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L47" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="n">
@@ -50265,6 +50459,9 @@
       <c r="K48" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L48" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="n">
@@ -50301,6 +50498,9 @@
       <c r="K49" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L49" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="n">
@@ -50337,6 +50537,9 @@
       <c r="K50" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L50" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="n">
@@ -50373,6 +50576,9 @@
       <c r="K51" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L51" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="n">
@@ -50407,6 +50613,9 @@
         <v>2.36</v>
       </c>
       <c r="K52" s="85" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="L52" s="85" t="n">
         <v>0</v>
       </c>
     </row>
@@ -50445,6 +50654,9 @@
       <c r="K53" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L53" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="n">
@@ -50481,6 +50693,9 @@
       <c r="K54" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L54" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="n">
@@ -50515,6 +50730,9 @@
         <v>0</v>
       </c>
       <c r="K55" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" s="85" t="n">
         <v>2.49</v>
       </c>
     </row>
@@ -50553,6 +50771,9 @@
       <c r="K56" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L56" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="n">
@@ -50589,6 +50810,9 @@
       <c r="K57" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L57" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="4" t="n">
@@ -50625,6 +50849,9 @@
       <c r="K58" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L58" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="n">
@@ -50659,6 +50886,9 @@
         <v>1.9</v>
       </c>
       <c r="K59" s="85" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="L59" s="85" t="n">
         <v>0</v>
       </c>
     </row>
@@ -50697,6 +50927,9 @@
       <c r="K60" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L60" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="4" t="n">
@@ -50733,6 +50966,9 @@
       <c r="K61" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L61" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="n">
@@ -50769,6 +51005,9 @@
       <c r="K62" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L62" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="n">
@@ -50803,6 +51042,9 @@
         <v>0.56043956</v>
       </c>
       <c r="K63" s="85" t="n">
+        <v>0.56043956</v>
+      </c>
+      <c r="L63" s="85" t="n">
         <v>0</v>
       </c>
     </row>
@@ -50841,6 +51083,9 @@
       <c r="K64" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L64" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="4" t="n">
@@ -50877,6 +51122,9 @@
       <c r="K65" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L65" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="n">
@@ -50913,6 +51161,9 @@
       <c r="K66" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L66" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="4" t="n">
@@ -50949,6 +51200,9 @@
       <c r="K67" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L67" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="4" t="n">
@@ -50983,6 +51237,9 @@
         <v>0</v>
       </c>
       <c r="K68" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L68" s="85" t="n">
         <v>0.142</v>
       </c>
     </row>
@@ -51019,6 +51276,9 @@
         <v>0.020622091</v>
       </c>
       <c r="K69" s="85" t="n">
+        <v>0.247257862</v>
+      </c>
+      <c r="L69" s="85" t="n">
         <v>0</v>
       </c>
     </row>
@@ -51057,6 +51317,9 @@
       <c r="K70" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L70" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="4" t="n">
@@ -51093,6 +51356,9 @@
       <c r="K71" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L71" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="4" t="n">
@@ -51129,6 +51395,9 @@
       <c r="K72" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L72" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="4" t="n">
@@ -51163,6 +51432,9 @@
         <v>0</v>
       </c>
       <c r="K73" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" s="85" t="n">
         <v>0.52</v>
       </c>
     </row>
@@ -51201,6 +51473,9 @@
       <c r="K74" s="85" t="n">
         <v>0</v>
       </c>
+      <c r="L74" s="85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="4" t="n">
@@ -51235,6 +51510,9 @@
         <v>0</v>
       </c>
       <c r="K75" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L75" s="85" t="n">
         <v>0.56</v>
       </c>
     </row>
@@ -51271,12 +51549,15 @@
         <v>0</v>
       </c>
       <c r="K76" s="85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L76" s="85" t="n">
         <v>1.32</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B78" s="62" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="C78" s="82" t="n">
         <f aca="false">SUMPRODUCT('Food Data'!$I$6:$I$76,C6:C76)</f>
@@ -51312,6 +51593,10 @@
       </c>
       <c r="K78" s="82" t="n">
         <f aca="false">SUMPRODUCT('Food Data'!$I$6:$I$76,K6:K76)</f>
+        <v>3.20470929168484</v>
+      </c>
+      <c r="L78" s="82" t="n">
+        <f aca="false">SUMPRODUCT('Food Data'!$I$6:$I$76,L6:L76)</f>
         <v>6.89354343509816</v>
       </c>
     </row>
@@ -51353,12 +51638,16 @@
       </c>
       <c r="K79" s="86" t="n">
         <f aca="false">K78*7</f>
+        <v>22.4329650417939</v>
+      </c>
+      <c r="L79" s="86" t="n">
+        <f aca="false">L78*7</f>
         <v>48.2548040456871</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="3" t="s">
-        <v>721</v>
+        <v>725</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51366,7 +51655,7 @@
         <v>34</v>
       </c>
       <c r="C82" s="87" t="n">
-        <f aca="false" t="array" ref="C82:K92">MMULT('Matrix Model'!F20:BX30,C6:K76)</f>
+        <f aca="false" t="array" ref="C82:L92">MMULT('Matrix Model'!F20:BX30,C6:L76)</f>
         <v>2878.500000161</v>
       </c>
       <c r="D82" s="87" t="n">
@@ -51391,6 +51680,9 @@
         <v>2878.500000161</v>
       </c>
       <c r="K82" s="87" t="n">
+        <v>2878.499999899</v>
+      </c>
+      <c r="L82" s="87" t="n">
         <v>2948.364</v>
       </c>
     </row>
@@ -51423,6 +51715,9 @@
         <v>111.99999999498</v>
       </c>
       <c r="K83" s="87" t="n">
+        <v>111.99999999639</v>
+      </c>
+      <c r="L83" s="87" t="n">
         <v>109.1001</v>
       </c>
     </row>
@@ -51455,6 +51750,9 @@
         <v>467.75624997971</v>
       </c>
       <c r="K84" s="87" t="n">
+        <v>466.48972753668</v>
+      </c>
+      <c r="L84" s="87" t="n">
         <v>361.76432</v>
       </c>
     </row>
@@ -51487,6 +51785,9 @@
         <v>66.16013141328</v>
       </c>
       <c r="K85" s="87" t="n">
+        <v>63.96666665434</v>
+      </c>
+      <c r="L85" s="87" t="n">
         <v>117.84292</v>
       </c>
     </row>
@@ -51519,6 +51820,9 @@
         <v>47.9185550492</v>
       </c>
       <c r="K86" s="87" t="n">
+        <v>48.2220552157</v>
+      </c>
+      <c r="L86" s="87" t="n">
         <v>14.415</v>
       </c>
     </row>
@@ -51551,6 +51855,9 @@
         <v>66.95184296326</v>
       </c>
       <c r="K87" s="87" t="n">
+        <v>60.39226110143</v>
+      </c>
+      <c r="L87" s="87" t="n">
         <v>89.91342</v>
       </c>
     </row>
@@ -51583,6 +51890,9 @@
         <v>999.999999987</v>
       </c>
       <c r="K88" s="87" t="n">
+        <v>1000.000000003</v>
+      </c>
+      <c r="L88" s="87" t="n">
         <v>1447.908</v>
       </c>
     </row>
@@ -51615,6 +51925,9 @@
         <v>23.30780114899</v>
       </c>
       <c r="K89" s="87" t="n">
+        <v>24.41683761813</v>
+      </c>
+      <c r="L89" s="87" t="n">
         <v>20.04404</v>
       </c>
     </row>
@@ -51647,6 +51960,9 @@
         <v>5247.643061918</v>
       </c>
       <c r="K90" s="87" t="n">
+        <v>5104.772296647</v>
+      </c>
+      <c r="L90" s="87" t="n">
         <v>2939.528</v>
       </c>
     </row>
@@ -51679,6 +51995,9 @@
         <v>768.584133897</v>
       </c>
       <c r="K91" s="87" t="n">
+        <v>572.38272993</v>
+      </c>
+      <c r="L91" s="87" t="n">
         <v>3856.936</v>
       </c>
     </row>
@@ -51711,17 +52030,20 @@
         <v>166.1430651884</v>
       </c>
       <c r="K92" s="87" t="n">
+        <v>166.134565981</v>
+      </c>
+      <c r="L92" s="87" t="n">
         <v>96.552</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>722</v>
+        <v>726</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B95" s="4" t="s">
-        <v>723</v>
+        <v>727</v>
       </c>
       <c r="C95" s="75" t="str">
         <f aca="false">IF(OR(C82&lt;3030*0.95-0.5,C82&gt;3030*1.05+0.5),"MISSED","ok")</f>
@@ -51759,10 +52081,14 @@
         <f aca="false">IF(OR(K82&lt;3030*0.95-0.5,K82&gt;3030*1.05+0.5),"MISSED","ok")</f>
         <v>ok</v>
       </c>
+      <c r="L95" s="75" t="str">
+        <f aca="false">IF(OR(L82&lt;3030*0.95-0.5,L82&gt;3030*1.05+0.5),"MISSED","ok")</f>
+        <v>ok</v>
+      </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B96" s="4" t="s">
-        <v>724</v>
+        <v>728</v>
       </c>
       <c r="C96" s="75" t="str">
         <f aca="false">IF(C83&lt;112-0.01,"MISSED","ok")</f>
@@ -51798,12 +52124,16 @@
       </c>
       <c r="K96" s="75" t="str">
         <f aca="false">IF(K83&lt;112-0.01,"MISSED","ok")</f>
+        <v>ok</v>
+      </c>
+      <c r="L96" s="75" t="str">
+        <f aca="false">IF(L83&lt;112-0.01,"MISSED","ok")</f>
         <v>MISSED</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B97" s="4" t="s">
-        <v>725</v>
+        <v>729</v>
       </c>
       <c r="C97" s="75" t="str">
         <f aca="false">IF(C86&lt;42-0.01,"MISSED","ok")</f>
@@ -51839,12 +52169,16 @@
       </c>
       <c r="K97" s="75" t="str">
         <f aca="false">IF(K86&lt;42-0.01,"MISSED","ok")</f>
+        <v>ok</v>
+      </c>
+      <c r="L97" s="75" t="str">
+        <f aca="false">IF(L86&lt;42-0.01,"MISSED","ok")</f>
         <v>MISSED</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B98" s="4" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C98" s="75" t="str">
         <f aca="false">IF(C88&lt;1000-0.01,"MISSED","ok")</f>
@@ -51882,10 +52216,14 @@
         <f aca="false">IF(K88&lt;1000-0.01,"MISSED","ok")</f>
         <v>ok</v>
       </c>
+      <c r="L98" s="75" t="str">
+        <f aca="false">IF(L88&lt;1000-0.01,"MISSED","ok")</f>
+        <v>ok</v>
+      </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B99" s="4" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="C99" s="75" t="str">
         <f aca="false">IF(C90&lt;3400-0.01,"MISSED","ok")</f>
@@ -51921,12 +52259,16 @@
       </c>
       <c r="K99" s="75" t="str">
         <f aca="false">IF(K90&lt;3400-0.01,"MISSED","ok")</f>
+        <v>ok</v>
+      </c>
+      <c r="L99" s="75" t="str">
+        <f aca="false">IF(L90&lt;3400-0.01,"MISSED","ok")</f>
         <v>MISSED</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B100" s="4" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="C100" s="75" t="str">
         <f aca="false">IF(C92&lt;90-0.01,"MISSED","ok")</f>
@@ -51964,10 +52306,14 @@
         <f aca="false">IF(K92&lt;90-0.01,"MISSED","ok")</f>
         <v>ok</v>
       </c>
+      <c r="L100" s="75" t="str">
+        <f aca="false">IF(L92&lt;90-0.01,"MISSED","ok")</f>
+        <v>ok</v>
+      </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B101" s="4" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
       <c r="C101" s="75" t="str">
         <f aca="false">IF(C91&gt;2300+0.01,"MISSED","ok")</f>
@@ -52003,12 +52349,16 @@
       </c>
       <c r="K101" s="75" t="str">
         <f aca="false">IF(K91&gt;2300+0.01,"MISSED","ok")</f>
+        <v>ok</v>
+      </c>
+      <c r="L101" s="75" t="str">
+        <f aca="false">IF(L91&gt;2300+0.01,"MISSED","ok")</f>
         <v>MISSED</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B102" s="4" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
       <c r="C102" s="75" t="str">
         <f aca="false">IF(C85*9&gt;C82*0.35+0.01,"MISSED","ok")</f>
@@ -52044,41 +52394,45 @@
       </c>
       <c r="K102" s="75" t="str">
         <f aca="false">IF(K85*9&gt;K82*0.35+0.01,"MISSED","ok")</f>
+        <v>ok</v>
+      </c>
+      <c r="L102" s="75" t="str">
+        <f aca="false">IF(L85*9&gt;L82*0.35+0.01,"MISSED","ok")</f>
         <v>MISSED</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="7" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="7" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="7" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="7" t="s">
-        <v>735</v>
+        <v>739</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="7" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C95:K102">
+  <conditionalFormatting sqref="C95:L102">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>C95="MISSED"</formula>
     </cfRule>
@@ -52099,7 +52453,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:BX74"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="14"/>
@@ -52107,38 +52461,38 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>737</v>
+        <v>741</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>739</v>
+        <v>743</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="F7" s="74" t="str">
         <f aca="false">'Matrix Model'!F13</f>
@@ -52427,10 +52781,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="B8" s="75" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="C8" s="78" t="n">
         <v>2878.5</v>
@@ -52722,10 +53076,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>747</v>
+        <v>751</v>
       </c>
       <c r="B9" s="75" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="C9" s="78" t="n">
         <v>112</v>
@@ -53017,10 +53371,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="B10" s="75" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="C10" s="78" t="n">
         <v>1000</v>
@@ -53312,10 +53666,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="B11" s="75" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="C11" s="78" t="n">
         <v>0</v>
@@ -53607,10 +53961,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
       <c r="B12" s="75" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="C12" s="78" t="n">
         <v>606</v>
@@ -53902,10 +54256,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>752</v>
+        <v>756</v>
       </c>
       <c r="B13" s="75" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="C13" s="78" t="n">
         <v>2.5</v>
@@ -54197,10 +54551,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="B14" s="75" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="C14" s="78" t="n">
         <v>2</v>
@@ -54492,10 +54846,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
+        <v>758</v>
+      </c>
+      <c r="B15" s="75" t="s">
         <v>754</v>
-      </c>
-      <c r="B15" s="75" t="s">
-        <v>750</v>
       </c>
       <c r="C15" s="78" t="n">
         <v>3</v>
@@ -54787,7 +55141,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="62" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="F17" s="88" t="n">
         <f aca="false">'Food Data'!I6</f>
@@ -55076,7 +55430,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="62" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
       <c r="F18" s="88" t="n">
         <f aca="false">'Diet Comparison'!C6</f>
@@ -55365,7 +55719,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="62" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="F19" s="88" t="n">
         <f aca="false">'Food Data'!N6*'Food Data'!P6/100</f>
@@ -55654,54 +56008,54 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>761</v>
+        <v>765</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>764</v>
+        <v>768</v>
       </c>
       <c r="H22" s="16" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="I22" s="16" t="s">
-        <v>766</v>
+        <v>770</v>
       </c>
       <c r="K22" s="89" t="s">
-        <v>767</v>
+        <v>771</v>
       </c>
       <c r="L22" s="89" t="s">
-        <v>768</v>
+        <v>772</v>
       </c>
       <c r="M22" s="89" t="s">
-        <v>769</v>
+        <v>773</v>
       </c>
       <c r="N22" s="89" t="s">
-        <v>770</v>
+        <v>774</v>
       </c>
       <c r="P22" s="16" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="Q22" s="16" t="s">
-        <v>771</v>
+        <v>775</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -56195,7 +56549,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="15" t="s">
-        <v>772</v>
+        <v>776</v>
       </c>
       <c r="K32" s="90" t="n">
         <f aca="false">Y19</f>
@@ -56216,7 +56570,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>773</v>
+        <v>777</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -56462,7 +56816,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="14" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
       <c r="B44" s="94" t="n">
         <f aca="false">MDETERM(B23:I30)</f>
@@ -56475,16 +56829,16 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="16" t="s">
-        <v>775</v>
+        <v>779</v>
       </c>
       <c r="B46" s="16" t="s">
-        <v>776</v>
+        <v>780</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>777</v>
+        <v>781</v>
       </c>
       <c r="D46" s="16" t="s">
-        <v>778</v>
+        <v>782</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -56618,7 +56972,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="15" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
       <c r="B55" s="15" t="str">
         <f aca="false">IF(MAX(D47:D54)-MIN(D47:D54)&lt;0.000001,"✓ B⁻¹r reproduces the Simplex answer","✗ mismatch")</f>
@@ -56627,27 +56981,27 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="16" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
       <c r="B58" s="16" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="C58" s="16" t="s">
-        <v>781</v>
+        <v>785</v>
       </c>
       <c r="D58" s="16" t="s">
-        <v>782</v>
+        <v>786</v>
       </c>
       <c r="E58" s="16" t="s">
-        <v>783</v>
+        <v>787</v>
       </c>
       <c r="G58" s="15" t="s">
-        <v>784</v>
+        <v>788</v>
       </c>
       <c r="H58" s="98" t="n">
         <f aca="false">U17</f>
@@ -56704,7 +57058,7 @@
         <v>$0.023 per +100 kcal</v>
       </c>
       <c r="G59" s="15" t="s">
-        <v>785</v>
+        <v>789</v>
       </c>
       <c r="H59" s="93" t="n">
         <f aca="false" t="array" ref="H59:O59">MMULT(H58:O58,B35:I42)</f>
@@ -56888,12 +57242,12 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="62" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
       <c r="F69" s="100" t="n">
         <f aca="false" t="array" ref="F69:BX69">F17:BX17-MMULT(H59:O59,F8:BX15)</f>
@@ -57112,225 +57466,225 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="62" t="s">
-        <v>788</v>
+        <v>792</v>
       </c>
       <c r="F70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="G70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="H70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="I70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="J70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="K70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="L70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="M70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="N70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="O70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="P70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="Q70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="R70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="S70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="T70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="U70" s="75" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="V70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="W70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="X70" s="75" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="Y70" s="75" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="Z70" s="75" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="AA70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AB70" s="75" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="AC70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AD70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AE70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AF70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AG70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AH70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AI70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AJ70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AK70" s="75" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="AL70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AM70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AN70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AO70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AP70" s="75" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="AQ70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AR70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AS70" s="75" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="AT70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AU70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AV70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AW70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AX70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AY70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="AZ70" s="75" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="BA70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BB70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BC70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BD70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BE70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BF70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BG70" s="75" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="BH70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BI70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BJ70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BK70" s="75" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="BL70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BM70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BN70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BO70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BP70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BQ70" s="75" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="BR70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BS70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BT70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BU70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BV70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BW70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="BX70" s="75" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="62" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="F71" s="75" t="str">
         <f aca="false">IF(F69&gt;=-0.000000001,"OK","FAIL")</f>
@@ -57619,12 +57973,12 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>793</v>
+        <v>797</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="101" t="s">
-        <v>794</v>
+        <v>798</v>
       </c>
       <c r="B74" s="101" t="str">
         <f aca="false">IF(AND(COUNTIF(F71:BX71,"FAIL")=0,COUNTIF(D59:D66,"✗")=0),"✓ PROVEN OPTIMAL: no food can be added, removed or swapped to lower the cost","✗ Not optimal for the current data — re-solve")</f>
@@ -57648,24 +58002,24 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:A34"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="150"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="102" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="103" t="s">
-        <v>796</v>
+        <v>800</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="103" t="s">
-        <v>797</v>
+        <v>801</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -57673,32 +58027,32 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="102" t="s">
-        <v>798</v>
+        <v>802</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="103" t="s">
-        <v>799</v>
+        <v>803</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="103" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="103" t="s">
-        <v>801</v>
+        <v>805</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="103" t="s">
-        <v>802</v>
+        <v>806</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="103" t="s">
-        <v>803</v>
+        <v>807</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -57706,47 +58060,47 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="102" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="103" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="103" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="103" t="s">
-        <v>807</v>
+        <v>811</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="103" t="s">
-        <v>808</v>
+        <v>812</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="103" t="s">
-        <v>809</v>
+        <v>813</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="103" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="103" t="s">
-        <v>811</v>
+        <v>815</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="103" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -57754,52 +58108,52 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="102" t="s">
-        <v>813</v>
+        <v>817</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="103" t="s">
-        <v>814</v>
+        <v>818</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="103" t="s">
-        <v>815</v>
+        <v>819</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="103" t="s">
-        <v>816</v>
+        <v>820</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="103" t="s">
-        <v>817</v>
+        <v>821</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="103" t="s">
-        <v>818</v>
+        <v>822</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="103" t="s">
-        <v>819</v>
+        <v>823</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="103" t="s">
-        <v>820</v>
+        <v>824</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="103" t="s">
-        <v>821</v>
+        <v>825</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="103" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -57807,12 +58161,12 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="102" t="s">
-        <v>823</v>
+        <v>827</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="103" t="s">
-        <v>824</v>
+        <v>828</v>
       </c>
     </row>
   </sheetData>

</xml_diff>